<commit_message>
Actualiza documentacion del proyecto
</commit_message>
<xml_diff>
--- a/Documentacion/Evidencias proyecto/Sprint Backlog/Sprint_Backlog_APT.xlsx
+++ b/Documentacion/Evidencias proyecto/Sprint Backlog/Sprint_Backlog_APT.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="1" r:id="Rdaa9a97ad67e47e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 2" sheetId="2" r:id="R01a93631a23a4709"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3" sheetId="3" r:id="R6f8ef2c4f2a14277"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4" sheetId="4" r:id="Re4c4e3e14c254a3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5" sheetId="5" r:id="R658d68c6f13a4c2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructivo" sheetId="6" r:id="R9b44c4cd91dc404d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="1" r:id="Rc6a2a9ae5b3944fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 2" sheetId="2" r:id="R9c645b2574d446b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3" sheetId="3" r:id="Rd0e38949052e4f71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4" sheetId="4" r:id="Rcbdd38a6b16e4b35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5" sheetId="5" r:id="R5be4ca3fdd5b409e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructivo" sheetId="6" r:id="R7132e8d5d290439a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -265,7 +265,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -276,7 +276,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -286,7 +286,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -297,7 +297,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -308,7 +308,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -318,7 +318,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -329,7 +329,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -340,7 +340,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -350,7 +350,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -361,7 +361,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -372,7 +372,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -382,7 +382,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -393,7 +393,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -404,7 +404,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -414,7 +414,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -425,7 +425,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -436,7 +436,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -446,7 +446,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -457,7 +457,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -468,7 +468,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -478,7 +478,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -489,7 +489,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -500,7 +500,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -510,7 +510,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -521,7 +521,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -532,7 +532,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -542,7 +542,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -553,7 +553,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -564,7 +564,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -574,7 +574,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -894,6 +894,7 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
+      <x:c r="E4"/>
       <x:c r="H4" s="25" t="str">
         <x:v>Día 1</x:v>
       </x:c>
@@ -941,10 +942,10 @@
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="B5" s="34" t="str">
-        <x:v>ID Product Backlog</x:v>
+        <x:v>ID Historia de Usuario</x:v>
       </x:c>
       <x:c r="C5" s="34" t="str">
-        <x:v>Enunciado del Product Backlog</x:v>
+        <x:v>Enunciado de la Historia de Usuario</x:v>
       </x:c>
       <x:c r="D5" s="34" t="str">
         <x:v>Tarea</x:v>
@@ -1036,7 +1037,7 @@
         <x:v>Definir flujo de autenticación, recuperación y permisos por rol</x:v>
       </x:c>
       <x:c r="E6" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F6" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -1130,7 +1131,7 @@
         <x:v>Configurar autenticación, sesiones y recuperación de contraseña en Django</x:v>
       </x:c>
       <x:c r="E7" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F7" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -1224,7 +1225,7 @@
         <x:v>Implementar endpoints de login, logout y recuperación de acceso</x:v>
       </x:c>
       <x:c r="E8" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F8" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -1506,7 +1507,7 @@
         <x:v>Ejecutar pruebas funcionales y de seguridad del acceso</x:v>
       </x:c>
       <x:c r="E11" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F11" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -1604,7 +1605,7 @@
         <x:v>Definir datos obligatorios y reglas de validación del registro</x:v>
       </x:c>
       <x:c r="E12" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F12" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -1698,7 +1699,7 @@
         <x:v>Implementar modelo, validaciones y endpoint de registro en Django</x:v>
       </x:c>
       <x:c r="E13" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F13" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -1980,7 +1981,7 @@
         <x:v>Probar duplicados, formatos, campos obligatorios y registro exitoso</x:v>
       </x:c>
       <x:c r="E16" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F16" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -2078,7 +2079,7 @@
         <x:v>Definir campos del perfil y reglas de privacidad de datos personales</x:v>
       </x:c>
       <x:c r="E17" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F17" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -2172,7 +2173,7 @@
         <x:v>Implementar consulta y actualización del perfil en Django</x:v>
       </x:c>
       <x:c r="E18" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F18" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -2360,7 +2361,7 @@
         <x:v>Integrar fecha de nacimiento y sector con la información de caracterización</x:v>
       </x:c>
       <x:c r="E20" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F20" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -2454,7 +2455,7 @@
         <x:v>Ejecutar pruebas de validación, edición y protección de datos</x:v>
       </x:c>
       <x:c r="E21" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F21" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -2552,7 +2553,7 @@
         <x:v>Modelar juntas, sectores y relaciones de asociación en MySQL/Django</x:v>
       </x:c>
       <x:c r="E22" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F22" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -2646,7 +2647,7 @@
         <x:v>Implementar CRUD y endpoints de juntas y sectores</x:v>
       </x:c>
       <x:c r="E23" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F23" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -2928,7 +2929,7 @@
         <x:v>Validar permisos y reglas de asociación territorial</x:v>
       </x:c>
       <x:c r="E26" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F26" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -3022,7 +3023,7 @@
         <x:v>Ejecutar pruebas de integración de juntas, sectores y usuarios</x:v>
       </x:c>
       <x:c r="E27" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F27" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -3108,6 +3109,45 @@
         <x:f>AA27</x:f>
         <x:v>4</x:v>
       </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="E28"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="E29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="E30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="E31"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="E32"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="E33"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="E34"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="E35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="E36"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="E37"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="E38"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="E39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="E40"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3268,6 +3308,7 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
+      <x:c r="E4"/>
       <x:c r="H4" s="25" t="str">
         <x:v>Día 1</x:v>
       </x:c>
@@ -3315,10 +3356,10 @@
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="B5" s="34" t="str">
-        <x:v>ID Product Backlog</x:v>
+        <x:v>ID Historia de Usuario</x:v>
       </x:c>
       <x:c r="C5" s="34" t="str">
-        <x:v>Enunciado del Product Backlog</x:v>
+        <x:v>Enunciado de la Historia de Usuario</x:v>
       </x:c>
       <x:c r="D5" s="34" t="str">
         <x:v>Tarea</x:v>
@@ -3404,13 +3445,13 @@
         <x:v>HU-05</x:v>
       </x:c>
       <x:c r="C6" s="63" t="str">
-        <x:v>Como usuario autorizado de gestión, quiero registrar a los integrantes previamente definidos de la directiva, asignar cargos y administrar roles o estados de usuario, para mantener los accesos y responsabilidades correctamente configurados sin realizar votaciones electrónicas.</x:v>
+        <x:v>Como administrador, quiero registrar a los integrantes previamente definidos de la directiva, asignar cargos y administrar roles o estados de usuario, para mantener los accesos y responsabilidades correctamente configurados sin realizar votaciones electrónicas.</x:v>
       </x:c>
       <x:c r="D6" s="64" t="str">
         <x:v>Modelar directiva, cargos, roles y estados de usuario</x:v>
       </x:c>
       <x:c r="E6" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F6" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -3504,7 +3545,7 @@
         <x:v>Implementar servicios y endpoints de gestión de cargos, roles y estados</x:v>
       </x:c>
       <x:c r="E7" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F7" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -3786,7 +3827,7 @@
         <x:v>Configurar y validar reglas de permisos asociadas a cargos y roles</x:v>
       </x:c>
       <x:c r="E10" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F10" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -3880,7 +3921,7 @@
         <x:v>Ejecutar pruebas de autorización, cambios de cargo y estados</x:v>
       </x:c>
       <x:c r="E11" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F11" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -3978,7 +4019,7 @@
         <x:v>Implementar modelo y API de publicaciones con almacenamiento local de archivos</x:v>
       </x:c>
       <x:c r="E12" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F12" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -4072,7 +4113,7 @@
         <x:v>Implementar modelo y servicio de notificaciones internas</x:v>
       </x:c>
       <x:c r="E13" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F13" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -4354,7 +4395,7 @@
         <x:v>Validar permisos, tipos de archivo y datos obligatorios</x:v>
       </x:c>
       <x:c r="E16" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F16" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -4448,7 +4489,7 @@
         <x:v>Ejecutar pruebas funcionales de publicaciones, adjuntos y alertas</x:v>
       </x:c>
       <x:c r="E17" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F17" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -4546,7 +4587,7 @@
         <x:v>Implementar modelo y API de actividades y eventos</x:v>
       </x:c>
       <x:c r="E18" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F18" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -4640,7 +4681,7 @@
         <x:v>Implementar reglas de fecha, estado, aforo y cancelación</x:v>
       </x:c>
       <x:c r="E19" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F19" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -4922,7 +4963,7 @@
         <x:v>Ejecutar pruebas backend de reglas y validaciones de eventos</x:v>
       </x:c>
       <x:c r="E22" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F22" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -5016,7 +5057,7 @@
         <x:v>Ejecutar pruebas funcionales y de aceptación del módulo</x:v>
       </x:c>
       <x:c r="E23" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F23" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -5114,7 +5155,7 @@
         <x:v>Implementar modelo y endpoint de inscripción a eventos</x:v>
       </x:c>
       <x:c r="E24" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F24" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -5208,7 +5249,7 @@
         <x:v>Implementar validación de cupos e inscripción duplicada</x:v>
       </x:c>
       <x:c r="E25" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F25" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -5490,7 +5531,7 @@
         <x:v>Probar cupos, duplicados, permisos y escenarios límite</x:v>
       </x:c>
       <x:c r="E28" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F28" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -5576,6 +5617,42 @@
         <x:f>AA28</x:f>
         <x:v>6</x:v>
       </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="E29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="E30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="E31"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="E32"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="E33"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="E34"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="E35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="E36"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="E37"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="E38"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="E39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="E40"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5736,6 +5813,7 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
+      <x:c r="E4"/>
       <x:c r="H4" s="25" t="str">
         <x:v>Día 1</x:v>
       </x:c>
@@ -5783,10 +5861,10 @@
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="B5" s="34" t="str">
-        <x:v>ID Product Backlog</x:v>
+        <x:v>ID Historia de Usuario</x:v>
       </x:c>
       <x:c r="C5" s="34" t="str">
-        <x:v>Enunciado del Product Backlog</x:v>
+        <x:v>Enunciado de la Historia de Usuario</x:v>
       </x:c>
       <x:c r="D5" s="34" t="str">
         <x:v>Tarea</x:v>
@@ -5878,7 +5956,7 @@
         <x:v>Implementar consulta de inscritos y registro de asistencia</x:v>
       </x:c>
       <x:c r="E6" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F6" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -6066,7 +6144,7 @@
         <x:v>Implementar validaciones y permisos para modificar asistencia</x:v>
       </x:c>
       <x:c r="E8" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F8" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -6160,7 +6238,7 @@
         <x:v>Ejecutar pruebas de integración del control de participantes</x:v>
       </x:c>
       <x:c r="E9" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F9" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -6254,7 +6332,7 @@
         <x:v>Preparar datos de demostración para eventos y asistencia</x:v>
       </x:c>
       <x:c r="E10" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F10" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -6352,7 +6430,7 @@
         <x:v>Modelar categorías y registro de consultas, reclamos y solicitudes</x:v>
       </x:c>
       <x:c r="E11" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F11" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -6446,7 +6524,7 @@
         <x:v>Implementar endpoint para crear solicitudes vecinales</x:v>
       </x:c>
       <x:c r="E12" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F12" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -6728,7 +6806,7 @@
         <x:v>Ejecutar pruebas de validación, seguridad y envío exitoso</x:v>
       </x:c>
       <x:c r="E15" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F15" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -6826,7 +6904,7 @@
         <x:v>Implementar flujo de estados e historial de cambios de solicitudes</x:v>
       </x:c>
       <x:c r="E16" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F16" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -6920,7 +6998,7 @@
         <x:v>Implementar APIs de listado, detalle, asignación y actualización</x:v>
       </x:c>
       <x:c r="E17" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F17" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -7202,7 +7280,7 @@
         <x:v>Probar permisos, historial y trazabilidad de cambios</x:v>
       </x:c>
       <x:c r="E20" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F20" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -7296,7 +7374,7 @@
         <x:v>Ejecutar pruebas funcionales de gestión completa de solicitudes</x:v>
       </x:c>
       <x:c r="E21" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F21" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -7394,7 +7472,7 @@
         <x:v>Modelar tipos, estados y solicitudes de documentos</x:v>
       </x:c>
       <x:c r="E22" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F22" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -7488,7 +7566,7 @@
         <x:v>Implementar APIs de solicitud, revisión, aprobación y archivo local</x:v>
       </x:c>
       <x:c r="E23" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F23" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -7770,7 +7848,7 @@
         <x:v>Probar permisos, archivos y descarga autorizada</x:v>
       </x:c>
       <x:c r="E26" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F26" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -7864,7 +7942,7 @@
         <x:v>Ejecutar pruebas funcionales del flujo documental</x:v>
       </x:c>
       <x:c r="E27" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F27" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -7962,7 +8040,7 @@
         <x:v>Implementar consulta consolidada de estado e historial del vecino</x:v>
       </x:c>
       <x:c r="E28" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F28" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -8056,7 +8134,7 @@
         <x:v>Implementar lógica de cambios no revisados y nuevas respuestas</x:v>
       </x:c>
       <x:c r="E29" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F29" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -8338,7 +8416,7 @@
         <x:v>Probar privacidad, estados, historial y acceso solo al propietario</x:v>
       </x:c>
       <x:c r="E32" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F32" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -8424,6 +8502,30 @@
         <x:f>AA32</x:f>
         <x:v>4</x:v>
       </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="E33"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="E34"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="E35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="E36"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="E37"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="E38"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="E39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="E40"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -8584,6 +8686,7 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
+      <x:c r="E4"/>
       <x:c r="H4" s="25" t="str">
         <x:v>Día 1</x:v>
       </x:c>
@@ -8631,10 +8734,10 @@
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="B5" s="34" t="str">
-        <x:v>ID Product Backlog</x:v>
+        <x:v>ID Historia de Usuario</x:v>
       </x:c>
       <x:c r="C5" s="34" t="str">
-        <x:v>Enunciado del Product Backlog</x:v>
+        <x:v>Enunciado de la Historia de Usuario</x:v>
       </x:c>
       <x:c r="D5" s="34" t="str">
         <x:v>Tarea</x:v>
@@ -8726,7 +8829,7 @@
         <x:v>Modelar conversaciones, mensajes y estados de lectura</x:v>
       </x:c>
       <x:c r="E6" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F6" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -8820,7 +8923,7 @@
         <x:v>Implementar APIs de bandeja, conversación, envío y lectura</x:v>
       </x:c>
       <x:c r="E7" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F7" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -9102,7 +9205,7 @@
         <x:v>Probar permisos y privacidad de las conversaciones</x:v>
       </x:c>
       <x:c r="E10" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F10" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -9196,7 +9299,7 @@
         <x:v>Ejecutar pruebas funcionales de envío y recepción de mensajes</x:v>
       </x:c>
       <x:c r="E11" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F11" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -9294,7 +9397,7 @@
         <x:v>Finalizar modelo de datos demográficos y reglas de privacidad</x:v>
       </x:c>
       <x:c r="E12" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F12" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -9388,7 +9491,7 @@
         <x:v>Implementar APIs de registro y consulta agregada de caracterización</x:v>
       </x:c>
       <x:c r="E13" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F13" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -9670,7 +9773,7 @@
         <x:v>Ejecutar pruebas de validación, anonimización y permisos</x:v>
       </x:c>
       <x:c r="E16" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F16" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -9764,7 +9867,7 @@
         <x:v>Preparar conjunto de datos sintéticos para demostración</x:v>
       </x:c>
       <x:c r="E17" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F17" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -9862,7 +9965,7 @@
         <x:v>Definir indicadores, fórmulas y reglas de cálculo</x:v>
       </x:c>
       <x:c r="E18" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F18" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -9956,7 +10059,7 @@
         <x:v>Implementar consultas de agregación y segmentación en MySQL/Django</x:v>
       </x:c>
       <x:c r="E19" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F19" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -10050,7 +10153,7 @@
         <x:v>Implementar servicio y endpoints de indicadores</x:v>
       </x:c>
       <x:c r="E20" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F20" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -10238,7 +10341,7 @@
         <x:v>Ejecutar pruebas de exactitud y consistencia de datos</x:v>
       </x:c>
       <x:c r="E22" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F22" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -10332,7 +10435,7 @@
         <x:v>Ejecutar pruebas básicas de rendimiento de consultas</x:v>
       </x:c>
       <x:c r="E23" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F23" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -10524,7 +10627,7 @@
         <x:v>Implementar endpoints agregados para el dashboard</x:v>
       </x:c>
       <x:c r="E25" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F25" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -10712,7 +10815,7 @@
         <x:v>Implementar generación de archivo de reporte agregado</x:v>
       </x:c>
       <x:c r="E27" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F27" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -10900,7 +11003,7 @@
         <x:v>Probar permisos y ámbito de datos de la junta</x:v>
       </x:c>
       <x:c r="E29" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F29" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -10994,7 +11097,7 @@
         <x:v>Validar consistencia de gráficos, indicadores y reporte exportado</x:v>
       </x:c>
       <x:c r="E30" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F30" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -11080,6 +11183,36 @@
         <x:f>AA30</x:f>
         <x:v>4</x:v>
       </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="E31"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="E32"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="E33"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="E34"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="E35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="E36"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="E37"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="E38"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="E39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="E40"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -11240,6 +11373,7 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
+      <x:c r="E4"/>
       <x:c r="H4" s="25" t="str">
         <x:v>Día 1</x:v>
       </x:c>
@@ -11287,10 +11421,10 @@
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="B5" s="34" t="str">
-        <x:v>ID Product Backlog</x:v>
+        <x:v>ID Historia de Usuario</x:v>
       </x:c>
       <x:c r="C5" s="34" t="str">
-        <x:v>Enunciado del Product Backlog</x:v>
+        <x:v>Enunciado de la Historia de Usuario</x:v>
       </x:c>
       <x:c r="D5" s="34" t="str">
         <x:v>Tarea</x:v>
@@ -11382,7 +11516,7 @@
         <x:v>Definir alcance de agregación municipal y permisos territoriales</x:v>
       </x:c>
       <x:c r="E6" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F6" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -11476,7 +11610,7 @@
         <x:v>Implementar APIs de agregación y comparación entre juntas y sectores</x:v>
       </x:c>
       <x:c r="E7" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F7" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -11758,7 +11892,7 @@
         <x:v>Implementar exportación de reportes municipales agregados</x:v>
       </x:c>
       <x:c r="E10" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F10" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -11852,7 +11986,7 @@
         <x:v>Ejecutar pruebas de privacidad y autorización municipal</x:v>
       </x:c>
       <x:c r="E11" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F11" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -11946,7 +12080,7 @@
         <x:v>Validar consistencia y rendimiento de datos consolidados</x:v>
       </x:c>
       <x:c r="E12" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F12" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -12040,7 +12174,7 @@
         <x:v>Preparar datos sintéticos de múltiples juntas para demostración</x:v>
       </x:c>
       <x:c r="E13" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F13" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -12138,7 +12272,7 @@
         <x:v>Implementar parámetros y consultas de filtrado en backend</x:v>
       </x:c>
       <x:c r="E14" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F14" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -12420,7 +12554,7 @@
         <x:v>Probar permisos, combinaciones sin resultados y restablecimiento</x:v>
       </x:c>
       <x:c r="E17" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F17" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -12514,7 +12648,7 @@
         <x:v>Ejecutar pruebas de integración y rendimiento de filtros</x:v>
       </x:c>
       <x:c r="E18" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F18" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -12606,13 +12740,13 @@
         <x:v>HU-19</x:v>
       </x:c>
       <x:c r="C19" s="63" t="str">
-        <x:v>Como vecino o integrante de la directiva, quiero consultar un chatbot de preguntas frecuentes, para recibir orientación rápida sobre la junta, actividades, publicaciones, documentos y uso de la plataforma.</x:v>
+        <x:v>Como usuario autorizado de la comunidad, quiero consultar un chatbot de preguntas frecuentes, para recibir orientación rápida sobre la junta de vecinos, actividades, publicaciones, documentos y uso de la plataforma.</x:v>
       </x:c>
       <x:c r="D19" s="64" t="str">
         <x:v>Definir alcance FAQ, reglas del prompt y política de seguridad</x:v>
       </x:c>
       <x:c r="E19" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F19" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -12706,7 +12840,7 @@
         <x:v>Integrar Gemini API gratuita desde el backend Django</x:v>
       </x:c>
       <x:c r="E20" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F20" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -12800,7 +12934,7 @@
         <x:v>Implementar servicio de contexto con información autorizada</x:v>
       </x:c>
       <x:c r="E21" s="65" t="str">
-        <x:v>Ivan Tamayo</x:v>
+        <x:v>Iván Tamayo</x:v>
       </x:c>
       <x:c r="F21" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -13082,7 +13216,7 @@
         <x:v>Ejecutar pruebas de privacidad, permisos y datos sensibles</x:v>
       </x:c>
       <x:c r="E24" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F24" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -13176,7 +13310,7 @@
         <x:v>Ejecutar pruebas funcionales de preguntas frecuentes</x:v>
       </x:c>
       <x:c r="E25" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F25" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -13270,7 +13404,7 @@
         <x:v>Preparar casos de demostración/fallback ante límites de la API</x:v>
       </x:c>
       <x:c r="E26" s="65" t="str">
-        <x:v>Richard Diaz</x:v>
+        <x:v>Richard Díaz</x:v>
       </x:c>
       <x:c r="F26" s="65" t="str">
         <x:v>Por iniciar</x:v>
@@ -13356,6 +13490,48 @@
         <x:f>AA26</x:f>
         <x:v>4</x:v>
       </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="E27"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="E28"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="E29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="E30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="E31"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="E32"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="E33"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="E34"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="E35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="E36"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="E37"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="E38"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="E39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="E40"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -13420,7 +13596,7 @@
     </x:row>
     <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="B4" s="60" t="str">
-        <x:v>Identificador (ID) de item de Product Backlog</x:v>
+        <x:v>Identificador (ID) de Historia de Usuario</x:v>
       </x:c>
       <x:c r="C4" s="60" t="str">
         <x:v>Código de la Historia de Usuario del Product Backlog a la cual pertenece la tarea.</x:v>
@@ -13428,10 +13604,10 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="B5" s="60" t="str">
-        <x:v>Enunciado del item de Product Backlog</x:v>
+        <x:v>Enunciado de la Historia de Usuario</x:v>
       </x:c>
       <x:c r="C5" s="60" t="str">
-        <x:v>Enunciado de la Historia de Usuario; se mantiene para conservar trazabilidad.</x:v>
+        <x:v>Enunciado oficial de la Historia de Usuario; se mantiene para conservar trazabilidad con el Product Backlog.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -13463,7 +13639,7 @@
         <x:v>Horas estimadas</x:v>
       </x:c>
       <x:c r="C9" s="60" t="str">
-        <x:v>Estimación inicial. Se usó como referencia académica 4 horas de esfuerzo de equipo por Story Point, distribuidas entre las tareas.</x:v>
+        <x:v>Estimación operativa inicial por tarea. Las horas sirven para planificar y dar seguimiento al trabajo del Sprint y se estiman de forma independiente de los Story Points; no existe una conversión fija entre Story Points y horas.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -13503,7 +13679,7 @@
         <x:v>Responsables</x:v>
       </x:c>
       <x:c r="C14" s="60" t="str">
-        <x:v>Ivan Tamayo: Scrum Master / Backend y Base de Datos. Rodrigo Romero: Frontend / UX-UI. Richard Diaz: Backend / QA y Pruebas.</x:v>
+        <x:v>Iván Tamayo: Scrum Master / Backend y Base de Datos. Rodrigo Romero: Frontend / UX-UI. Richard Díaz: Backend / QA y Pruebas.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">

</xml_diff>